<commit_message>
feat: default selected subject to teacher taught subjects and sync dashboard changes for production
</commit_message>
<xml_diff>
--- a/Data/LoginData.xlsx
+++ b/Data/LoginData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\panga\OneDrive\Desktop\Seva\SRSMA\SRSMADashBoard\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E05601C6-91CC-430E-AB89-E20E1BBC39D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DB84D5-6CCA-4C0F-A19C-E50F8A347FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="70">
   <si>
     <t>username</t>
   </si>
@@ -34,188 +34,212 @@
     <t>Role</t>
   </si>
   <si>
+    <t>Roll No</t>
+  </si>
+  <si>
+    <t>Abhinav</t>
+  </si>
+  <si>
+    <t>12+</t>
+  </si>
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>12+01</t>
+  </si>
+  <si>
+    <t>Abrar</t>
+  </si>
+  <si>
+    <t>12+02</t>
+  </si>
+  <si>
+    <t>Akhilesh</t>
+  </si>
+  <si>
+    <t>12+03</t>
+  </si>
+  <si>
+    <t>Aniesh</t>
+  </si>
+  <si>
+    <t>12+04</t>
+  </si>
+  <si>
+    <t>Chandrahaas</t>
+  </si>
+  <si>
+    <t>12+05</t>
+  </si>
+  <si>
+    <t>Ishan</t>
+  </si>
+  <si>
+    <t>12+06</t>
+  </si>
+  <si>
+    <t>Jagat Pavitra</t>
+  </si>
+  <si>
+    <t>12+07</t>
+  </si>
+  <si>
+    <t>Karthik</t>
+  </si>
+  <si>
+    <t>12+08</t>
+  </si>
+  <si>
+    <t>Krishna</t>
+  </si>
+  <si>
+    <t>12+09</t>
+  </si>
+  <si>
+    <t>Manideep</t>
+  </si>
+  <si>
+    <t>12+10</t>
+  </si>
+  <si>
+    <t>Mubashshir</t>
+  </si>
+  <si>
+    <t>12+11</t>
+  </si>
+  <si>
+    <t>Puneeth</t>
+  </si>
+  <si>
+    <t>12+12</t>
+  </si>
+  <si>
     <t>Sumedh</t>
   </si>
   <si>
-    <t>12+</t>
-  </si>
-  <si>
-    <t>Student</t>
-  </si>
-  <si>
-    <t>Chandrahaas</t>
-  </si>
-  <si>
-    <t>Ishan</t>
-  </si>
-  <si>
-    <t>Mubashshir</t>
-  </si>
-  <si>
-    <t>Jagat Pavitra</t>
-  </si>
-  <si>
-    <t>Abrar</t>
-  </si>
-  <si>
-    <t>Akhilesh</t>
-  </si>
-  <si>
-    <t>Manideep</t>
-  </si>
-  <si>
-    <t>Karthik</t>
-  </si>
-  <si>
-    <t>Abhinav</t>
-  </si>
-  <si>
-    <t>Krishna</t>
+    <t>12+13</t>
   </si>
   <si>
     <t>Sushil</t>
   </si>
   <si>
-    <t>Puneeth</t>
-  </si>
-  <si>
-    <t>Aniesh</t>
+    <t>12+14</t>
+  </si>
+  <si>
+    <t>Tarun</t>
+  </si>
+  <si>
+    <t>12+15</t>
   </si>
   <si>
     <t>SRSMA</t>
   </si>
   <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>Adwait</t>
+  </si>
+  <si>
+    <t>Bhavya Sri</t>
+  </si>
+  <si>
+    <t>Chaitanya</t>
+  </si>
+  <si>
+    <t>Dhaval</t>
+  </si>
+  <si>
+    <t>Haripada</t>
+  </si>
+  <si>
+    <t>Harshit</t>
+  </si>
+  <si>
+    <t>Ishwarya</t>
+  </si>
+  <si>
+    <t>Jayasimha</t>
+  </si>
+  <si>
+    <t>Koushik</t>
+  </si>
+  <si>
+    <t>Lokesh D</t>
+  </si>
+  <si>
+    <t>Narahari</t>
+  </si>
+  <si>
+    <t>Pruthviraj</t>
+  </si>
+  <si>
+    <t>Puneet</t>
+  </si>
+  <si>
+    <t>Shivendra</t>
+  </si>
+  <si>
+    <t>Sony</t>
+  </si>
+  <si>
+    <t>Subhaang</t>
+  </si>
+  <si>
+    <t>Sukdev</t>
+  </si>
+  <si>
+    <t>Surya</t>
+  </si>
+  <si>
+    <t>Susen</t>
+  </si>
+  <si>
+    <t>Vaishali</t>
+  </si>
+  <si>
+    <t>Ved Sharma</t>
+  </si>
+  <si>
+    <t>Ninad</t>
+  </si>
+  <si>
+    <t>Nitai108</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Saurabh</t>
+  </si>
+  <si>
+    <t>Advaitha108</t>
+  </si>
+  <si>
+    <t>VTD</t>
+  </si>
+  <si>
+    <t>Gadhadhar108</t>
+  </si>
+  <si>
+    <t>SSD</t>
+  </si>
+  <si>
+    <t>Srivas108</t>
+  </si>
+  <si>
     <t>Teacher</t>
-  </si>
-  <si>
-    <t>Surya</t>
-  </si>
-  <si>
-    <t>Ishwarya</t>
-  </si>
-  <si>
-    <t>Bhavya Sri</t>
-  </si>
-  <si>
-    <t>Subhaang</t>
-  </si>
-  <si>
-    <t>Adwait</t>
-  </si>
-  <si>
-    <t>Chaitanya</t>
-  </si>
-  <si>
-    <t>Haripada</t>
-  </si>
-  <si>
-    <t>Pruthviraj</t>
-  </si>
-  <si>
-    <t>Ved Sharma</t>
-  </si>
-  <si>
-    <t>Jayasimha</t>
-  </si>
-  <si>
-    <t>Harshit</t>
-  </si>
-  <si>
-    <t>Dhaval</t>
-  </si>
-  <si>
-    <t>Lokesh D</t>
-  </si>
-  <si>
-    <t>Sukdev</t>
-  </si>
-  <si>
-    <t>Narahari</t>
-  </si>
-  <si>
-    <t>Sony</t>
-  </si>
-  <si>
-    <t>Puneet</t>
-  </si>
-  <si>
-    <t>Vaishali</t>
-  </si>
-  <si>
-    <t>Koushik</t>
-  </si>
-  <si>
-    <t>Shivendra</t>
-  </si>
-  <si>
-    <t>Susen</t>
-  </si>
-  <si>
-    <t>Tarun</t>
-  </si>
-  <si>
-    <t>Roll No</t>
-  </si>
-  <si>
-    <t>12+01</t>
-  </si>
-  <si>
-    <t>12+02</t>
-  </si>
-  <si>
-    <t>12+03</t>
-  </si>
-  <si>
-    <t>12+04</t>
-  </si>
-  <si>
-    <t>12+05</t>
-  </si>
-  <si>
-    <t>12+06</t>
-  </si>
-  <si>
-    <t>12+07</t>
-  </si>
-  <si>
-    <t>12+08</t>
-  </si>
-  <si>
-    <t>12+09</t>
-  </si>
-  <si>
-    <t>12+10</t>
-  </si>
-  <si>
-    <t>12+11</t>
-  </si>
-  <si>
-    <t>12+12</t>
-  </si>
-  <si>
-    <t>12+13</t>
-  </si>
-  <si>
-    <t>12+14</t>
-  </si>
-  <si>
-    <t>12+15</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -582,12 +606,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="3" max="3" width="4.796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -603,278 +623,278 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <v>12345</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>12345</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>12345</v>
       </c>
       <c r="C4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>12345</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B6">
         <v>12345</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B7">
         <v>12345</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>12345</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>12345</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B10">
         <v>12345</v>
       </c>
       <c r="C10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B11">
         <v>12345</v>
       </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B12">
         <v>12345</v>
       </c>
       <c r="C12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="B13">
         <v>12345</v>
       </c>
       <c r="C13" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>12345</v>
       </c>
       <c r="C14" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D14" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" t="s">
-        <v>57</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="B15">
         <v>12345</v>
       </c>
       <c r="C15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B16">
         <v>12345</v>
       </c>
       <c r="C16" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="B17">
         <v>12345</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="B18">
         <v>12345</v>
@@ -883,7 +903,7 @@
         <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E18">
         <v>1201</v>
@@ -891,7 +911,7 @@
     </row>
     <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B19">
         <v>12345</v>
@@ -900,7 +920,7 @@
         <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E19">
         <v>1202</v>
@@ -908,7 +928,7 @@
     </row>
     <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="B20">
         <v>12345</v>
@@ -917,7 +937,7 @@
         <v>12</v>
       </c>
       <c r="D20" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E20">
         <v>1203</v>
@@ -925,7 +945,7 @@
     </row>
     <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B21">
         <v>12345</v>
@@ -934,7 +954,7 @@
         <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21">
         <v>1204</v>
@@ -942,7 +962,7 @@
     </row>
     <row r="22" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="B22">
         <v>12345</v>
@@ -951,7 +971,7 @@
         <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E22">
         <v>1205</v>
@@ -959,7 +979,7 @@
     </row>
     <row r="23" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="B23">
         <v>12345</v>
@@ -968,7 +988,7 @@
         <v>12</v>
       </c>
       <c r="D23" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E23">
         <v>1206</v>
@@ -976,7 +996,7 @@
     </row>
     <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B24">
         <v>12345</v>
@@ -985,7 +1005,7 @@
         <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E24">
         <v>1207</v>
@@ -993,7 +1013,7 @@
     </row>
     <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="B25">
         <v>12345</v>
@@ -1002,7 +1022,7 @@
         <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E25">
         <v>1208</v>
@@ -1010,7 +1030,7 @@
     </row>
     <row r="26" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B26">
         <v>12345</v>
@@ -1019,7 +1039,7 @@
         <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E26">
         <v>1209</v>
@@ -1027,7 +1047,7 @@
     </row>
     <row r="27" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B27">
         <v>12345</v>
@@ -1036,7 +1056,7 @@
         <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E27">
         <v>1210</v>
@@ -1044,7 +1064,7 @@
     </row>
     <row r="28" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="B28">
         <v>12345</v>
@@ -1053,7 +1073,7 @@
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E28">
         <v>1211</v>
@@ -1061,7 +1081,7 @@
     </row>
     <row r="29" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="B29">
         <v>12345</v>
@@ -1070,7 +1090,7 @@
         <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E29">
         <v>1212</v>
@@ -1078,7 +1098,7 @@
     </row>
     <row r="30" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="B30">
         <v>12345</v>
@@ -1087,7 +1107,7 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E30">
         <v>1213</v>
@@ -1095,7 +1115,7 @@
     </row>
     <row r="31" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="B31">
         <v>12345</v>
@@ -1104,7 +1124,7 @@
         <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E31">
         <v>1214</v>
@@ -1112,7 +1132,7 @@
     </row>
     <row r="32" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="B32">
         <v>12345</v>
@@ -1121,7 +1141,7 @@
         <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32">
         <v>1215</v>
@@ -1129,7 +1149,7 @@
     </row>
     <row r="33" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="B33">
         <v>12345</v>
@@ -1138,7 +1158,7 @@
         <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E33">
         <v>1216</v>
@@ -1146,7 +1166,7 @@
     </row>
     <row r="34" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="B34">
         <v>12345</v>
@@ -1155,7 +1175,7 @@
         <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E34">
         <v>1217</v>
@@ -1163,7 +1183,7 @@
     </row>
     <row r="35" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="B35">
         <v>12345</v>
@@ -1172,7 +1192,7 @@
         <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E35">
         <v>1218</v>
@@ -1180,7 +1200,7 @@
     </row>
     <row r="36" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="B36">
         <v>12345</v>
@@ -1189,7 +1209,7 @@
         <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E36">
         <v>1219</v>
@@ -1197,7 +1217,7 @@
     </row>
     <row r="37" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="B37">
         <v>12345</v>
@@ -1206,7 +1226,7 @@
         <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E37">
         <v>1220</v>
@@ -1214,7 +1234,7 @@
     </row>
     <row r="38" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="B38">
         <v>12345</v>
@@ -1223,21 +1243,72 @@
         <v>12</v>
       </c>
       <c r="D38" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E38">
         <v>1221</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15.6" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>60</v>
+      </c>
+      <c r="B39" t="s">
+        <v>61</v>
+      </c>
+      <c r="C39" t="s">
+        <v>62</v>
+      </c>
+      <c r="D39" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40" t="s">
+        <v>64</v>
+      </c>
+      <c r="C40" t="s">
+        <v>62</v>
+      </c>
+      <c r="D40" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B41" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" t="s">
+        <v>62</v>
+      </c>
+      <c r="D41" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C42" t="s">
+        <v>62</v>
+      </c>
+      <c r="D42" t="s">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A18:E38">
-    <sortCondition ref="A18:A38"/>
-  </sortState>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A17:D17" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E38 A40:C42 A39:C39 E39 E40:E42" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>